<commit_message>
Add Recoome & guldo
</commit_message>
<xml_diff>
--- a/EZAStatCalculator.xlsx
+++ b/EZAStatCalculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tyler\Documents\DokkanAnalysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61201ECA-33FB-433E-B7A5-F1A5EDF1A3EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95533159-2A28-4B2E-9E83-9C9EDF60BC1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11168" yWindow="0" windowWidth="11415" windowHeight="14362" xr2:uid="{BAE61A90-60AD-488C-ADA9-AC7F6409FE0C}"/>
+    <workbookView xWindow="11085" yWindow="0" windowWidth="11415" windowHeight="14280" xr2:uid="{BAE61A90-60AD-488C-ADA9-AC7F6409FE0C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -457,14 +457,14 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>3961</v>
+        <v>2716</v>
       </c>
       <c r="C3">
-        <v>13074</v>
+        <v>8966</v>
       </c>
       <c r="D3">
         <f>ROUND(C3+0.4839*(C3-B3),0)</f>
-        <v>17484</v>
+        <v>11990</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
@@ -472,14 +472,14 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>2243</v>
+        <v>2180</v>
       </c>
       <c r="C4">
-        <v>7403</v>
+        <v>7197</v>
       </c>
       <c r="D4">
         <f t="shared" ref="D4:D5" si="0">ROUND(C4+0.4839*(C4-B4),0)</f>
-        <v>9900</v>
+        <v>9625</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
@@ -487,14 +487,14 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>1512</v>
+        <v>2212</v>
       </c>
       <c r="C5">
-        <v>4990</v>
+        <v>7301</v>
       </c>
       <c r="D5">
         <f t="shared" si="0"/>
-        <v>6673</v>
+        <v>9764</v>
       </c>
     </row>
   </sheetData>
@@ -502,5 +502,6 @@
     <mergeCell ref="B1:D1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add EZA Captain Ginyu
</commit_message>
<xml_diff>
--- a/EZAStatCalculator.xlsx
+++ b/EZAStatCalculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tyler\Documents\DokkanAnalysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95533159-2A28-4B2E-9E83-9C9EDF60BC1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6E17F43-13AB-4635-9AF4-CB2D3C1ACA8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11085" yWindow="0" windowWidth="11415" windowHeight="14280" xr2:uid="{BAE61A90-60AD-488C-ADA9-AC7F6409FE0C}"/>
+    <workbookView xWindow="11168" yWindow="0" windowWidth="11415" windowHeight="14362" xr2:uid="{BAE61A90-60AD-488C-ADA9-AC7F6409FE0C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -457,14 +457,14 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>2716</v>
+        <v>4440</v>
       </c>
       <c r="C3">
-        <v>8966</v>
+        <v>14655</v>
       </c>
       <c r="D3">
         <f>ROUND(C3+0.4839*(C3-B3),0)</f>
-        <v>11990</v>
+        <v>19598</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
@@ -472,14 +472,14 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>2180</v>
+        <v>2855</v>
       </c>
       <c r="C4">
-        <v>7197</v>
+        <v>9423</v>
       </c>
       <c r="D4">
         <f t="shared" ref="D4:D5" si="0">ROUND(C4+0.4839*(C4-B4),0)</f>
-        <v>9625</v>
+        <v>12601</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
@@ -487,14 +487,14 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>2212</v>
+        <v>1691</v>
       </c>
       <c r="C5">
-        <v>7301</v>
+        <v>5582</v>
       </c>
       <c r="D5">
         <f t="shared" si="0"/>
-        <v>9764</v>
+        <v>7465</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
INT 19 & 20 EZA
</commit_message>
<xml_diff>
--- a/EZAStatCalculator.xlsx
+++ b/EZAStatCalculator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tyler\Documents\DokkanAnalysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{854807A7-85F5-4206-A6A2-5AA6C004D62D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B9ABADC-6941-4B9A-A238-751DC09A5452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-83" yWindow="0" windowWidth="11415" windowHeight="14362" xr2:uid="{BAE61A90-60AD-488C-ADA9-AC7F6409FE0C}"/>
   </bookViews>
@@ -457,14 +457,14 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>3171</v>
+        <v>2063</v>
       </c>
       <c r="C3">
-        <v>10465</v>
+        <v>6809</v>
       </c>
       <c r="D3">
         <f>ROUND(C3+0.4839*(C3-B3),0)</f>
-        <v>13995</v>
+        <v>9106</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
@@ -472,14 +472,14 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>3767</v>
+        <v>2803</v>
       </c>
       <c r="C4">
-        <v>12432</v>
+        <v>9251</v>
       </c>
       <c r="D4">
         <f t="shared" ref="D4:D5" si="0">ROUND(C4+0.4839*(C4-B4),0)</f>
-        <v>16625</v>
+        <v>12371</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
@@ -487,14 +487,14 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>1925</v>
+        <v>1760</v>
       </c>
       <c r="C5">
-        <v>6353</v>
+        <v>5811</v>
       </c>
       <c r="D5">
         <f t="shared" si="0"/>
-        <v>8496</v>
+        <v>7771</v>
       </c>
     </row>
   </sheetData>

</xml_diff>